<commit_message>
Add set_to compatibility and profiling data
</commit_message>
<xml_diff>
--- a/client-env/profiling/client_profiling.xlsx
+++ b/client-env/profiling/client_profiling.xlsx
@@ -8,26 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\client-env\profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551C7990-A89A-4A7D-91C6-C9E4616F48A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9DE080-1ACA-4751-B326-FFC2EF0D8BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test_connection" sheetId="1" r:id="rId1"/>
-    <sheet name="set" sheetId="2" r:id="rId2"/>
-    <sheet name="get" sheetId="3" r:id="rId3"/>
-    <sheet name="get_range" sheetId="4" r:id="rId4"/>
-    <sheet name="del_keys" sheetId="5" r:id="rId5"/>
-    <sheet name="del_values" sheetId="6" r:id="rId6"/>
-    <sheet name="2.Profiling" sheetId="7" r:id="rId7"/>
-    <sheet name="3. Profiling" sheetId="8" r:id="rId8"/>
+    <sheet name="set_single" sheetId="9" r:id="rId2"/>
+    <sheet name="set" sheetId="2" r:id="rId3"/>
+    <sheet name="get" sheetId="3" r:id="rId4"/>
+    <sheet name="get_range" sheetId="4" r:id="rId5"/>
+    <sheet name="del_keys" sheetId="5" r:id="rId6"/>
+    <sheet name="del_values" sheetId="6" r:id="rId7"/>
+    <sheet name="2.Profiling" sheetId="7" r:id="rId8"/>
+    <sheet name="3. Profiling" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="30">
   <si>
     <t>Middleware_Server: 10.0.2.87 (zs07)</t>
   </si>
@@ -114,6 +115,9 @@
   </si>
   <si>
     <t>Configs: VIRTUAL_SITES = 5</t>
+  </si>
+  <si>
+    <t>Total_Time [Initial]_[Connection_Setup]</t>
   </si>
 </sst>
 </file>
@@ -347,7 +351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -379,8 +383,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -388,6 +390,9 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -705,7 +710,7 @@
   <dimension ref="A1:Q84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.42578125" customWidth="1"/>
+    <col min="1" max="1" width="39" customWidth="1"/>
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
     <col min="3" max="3" width="33.5703125" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
@@ -738,47 +743,47 @@
       <c r="A6" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="27" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="25"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="27">
+      <c r="A7" s="33">
         <v>1</v>
       </c>
-      <c r="B7" s="31">
-        <v>0</v>
-      </c>
-      <c r="C7" s="31">
-        <v>5.1743999356403904E-3</v>
+      <c r="B7" s="29">
+        <v>7.0000533014535904E-7</v>
+      </c>
+      <c r="C7" s="29">
+        <v>6.2809999799355804E-3</v>
       </c>
       <c r="D7" s="21"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="27">
+      <c r="A8" s="33">
         <v>10</v>
       </c>
-      <c r="B8" s="31">
-        <v>0</v>
-      </c>
-      <c r="C8" s="33">
-        <v>8.2283001393079703E-4</v>
+      <c r="B8" s="29">
+        <v>3.2000243663787799E-6</v>
+      </c>
+      <c r="C8" s="31">
+        <v>2.9709199909120701E-2</v>
       </c>
       <c r="D8" s="22"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="27">
+      <c r="A9" s="33">
         <v>100</v>
       </c>
-      <c r="B9" s="31">
-        <v>0</v>
-      </c>
-      <c r="C9" s="31">
-        <v>5.3790500271134003E-4</v>
+      <c r="B9" s="29">
+        <v>2.06999247893691E-5</v>
+      </c>
+      <c r="C9" s="29">
+        <v>0.24735639989375999</v>
       </c>
       <c r="D9" s="21"/>
       <c r="I9" s="20"/>
@@ -786,106 +791,107 @@
       <c r="Q9" s="2"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="27">
+      <c r="A10" s="33">
         <v>1000</v>
       </c>
-      <c r="B10" s="31">
-        <v>0</v>
-      </c>
-      <c r="C10" s="31">
-        <v>3.6490820092149E-4</v>
+      <c r="B10" s="29">
+        <v>5.5799959227442701E-5</v>
+      </c>
+      <c r="C10" s="29">
+        <v>2.4106429001549201</v>
       </c>
       <c r="D10" s="23"/>
       <c r="H10" s="20"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="27">
-        <v>10000</v>
-      </c>
-      <c r="B11" s="31">
-        <v>0</v>
-      </c>
-      <c r="C11" s="31">
-        <v>3.3099438004428498E-4</v>
-      </c>
+      <c r="A11" s="33"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
       <c r="D11" s="21"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="27"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31">
-        <v>0</v>
-      </c>
+      <c r="A12" s="33"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="23"/>
       <c r="E12" s="17"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="27"/>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31">
-        <v>0</v>
-      </c>
+      <c r="A13" s="33"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
       <c r="D13" s="21"/>
       <c r="E13" s="17"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="27"/>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31">
-        <v>0</v>
-      </c>
+      <c r="A14" s="33"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="21"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="28"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32">
-        <v>0</v>
-      </c>
+      <c r="A15" s="34"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
       <c r="D15" s="24"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="32"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="32"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="32"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="32" t="s">
+        <v>29</v>
+      </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="32">
+        <v>6.6191999940201597E-3</v>
+      </c>
       <c r="B20" s="4"/>
       <c r="C20" s="3"/>
       <c r="D20" s="17"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="32"/>
       <c r="B21" s="4"/>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="32"/>
       <c r="B22" s="4"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="32"/>
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="32"/>
       <c r="B24" s="5"/>
       <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="32"/>
       <c r="B25" s="4"/>
       <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="32"/>
       <c r="B26" s="4"/>
       <c r="C26" s="3"/>
     </row>
@@ -901,7 +907,7 @@
       <c r="B28" s="5"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="30">
+      <c r="A29" s="28">
         <v>2.08998244488611E-7</v>
       </c>
     </row>
@@ -1105,11 +1111,420 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{349D7314-AB8E-4AA0-A861-31CE52CA3EE8}">
+  <dimension ref="A1:Q84"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="39" customWidth="1"/>
+    <col min="2" max="2" width="37.85546875" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" customWidth="1"/>
+    <col min="4" max="4" width="23.85546875" customWidth="1"/>
+    <col min="5" max="5" width="35.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="25"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="33">
+        <v>1</v>
+      </c>
+      <c r="B7" s="29">
+        <v>0</v>
+      </c>
+      <c r="C7" s="29">
+        <v>0</v>
+      </c>
+      <c r="D7" s="21"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="33">
+        <v>10</v>
+      </c>
+      <c r="B8" s="29">
+        <v>0</v>
+      </c>
+      <c r="C8" s="31">
+        <v>0</v>
+      </c>
+      <c r="D8" s="22"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="33">
+        <v>100</v>
+      </c>
+      <c r="B9" s="29">
+        <v>0</v>
+      </c>
+      <c r="C9" s="29">
+        <v>0</v>
+      </c>
+      <c r="D9" s="21"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="Q9" s="2"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="33">
+        <v>1000</v>
+      </c>
+      <c r="B10" s="29">
+        <v>0</v>
+      </c>
+      <c r="C10" s="29">
+        <v>0</v>
+      </c>
+      <c r="D10" s="23"/>
+      <c r="H10" s="20"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="33"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="21"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="33"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="17"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" s="33"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="17"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" s="33"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="21"/>
+    </row>
+    <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="34"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="24"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="32"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="32"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="32"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="32">
+        <v>6.6191999940201597E-3</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="17"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="32"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="32"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="3"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="32"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="3"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="32"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="3"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="32"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="3"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="32"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="3"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="5"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="28">
+        <v>2.08998244488611E-7</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33" s="4"/>
+      <c r="C33" s="3"/>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" s="5"/>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" s="4"/>
+      <c r="C36" s="3"/>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="4"/>
+      <c r="C37" s="3"/>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B38" s="4"/>
+      <c r="C38" s="3"/>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B39" s="4"/>
+      <c r="C39" s="3"/>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B40" s="4"/>
+      <c r="C40" s="3"/>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B41" s="4"/>
+      <c r="C41" s="3"/>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B42" s="4"/>
+      <c r="C42" s="3"/>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B43" s="4"/>
+      <c r="C43" s="3"/>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B44" s="4"/>
+      <c r="C44" s="3"/>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B45" s="4"/>
+      <c r="C45" s="3"/>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B46" s="4"/>
+      <c r="C46" s="3"/>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B47" s="4"/>
+      <c r="C47" s="3"/>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B48" s="4"/>
+      <c r="C48" s="3"/>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" s="4"/>
+      <c r="C49" s="3"/>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50" s="4"/>
+      <c r="C50" s="3"/>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51" s="4"/>
+      <c r="C51" s="3"/>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B52" s="4"/>
+      <c r="C52" s="3"/>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B53" s="4"/>
+      <c r="C53" s="3"/>
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B54" s="4"/>
+      <c r="C54" s="3"/>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B55" s="4"/>
+      <c r="C55" s="3"/>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B56" s="4"/>
+      <c r="C56" s="3"/>
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B57" s="4"/>
+      <c r="C57" s="3"/>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B58" s="4"/>
+      <c r="C58" s="3"/>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B59" s="4"/>
+      <c r="C59" s="3"/>
+    </row>
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B60" s="4"/>
+      <c r="C60" s="3"/>
+    </row>
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B61" s="4"/>
+      <c r="C61" s="3"/>
+    </row>
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B62" s="4"/>
+      <c r="C62" s="3"/>
+    </row>
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B63" s="4"/>
+      <c r="C63" s="3"/>
+    </row>
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B64" s="4"/>
+      <c r="C64" s="3"/>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B65" s="4"/>
+      <c r="C65" s="3"/>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B66" s="4"/>
+      <c r="C66" s="3"/>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B67" s="4"/>
+      <c r="C67" s="3"/>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B68" s="4"/>
+      <c r="C68" s="3"/>
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B69" s="4"/>
+      <c r="C69" s="3"/>
+    </row>
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B70" s="4"/>
+      <c r="C70" s="3"/>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B71" s="4"/>
+      <c r="C71" s="3"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B72" s="4"/>
+      <c r="C72" s="3"/>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B73" s="4"/>
+      <c r="C73" s="3"/>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B74" s="4"/>
+      <c r="C74" s="3"/>
+    </row>
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B75" s="4"/>
+      <c r="C75" s="3"/>
+    </row>
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B76" s="4"/>
+      <c r="C76" s="1"/>
+    </row>
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C77" s="1"/>
+    </row>
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C78" s="1"/>
+    </row>
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C79" s="1"/>
+    </row>
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C80" s="1"/>
+    </row>
+    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C81" s="1"/>
+    </row>
+    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C82" s="1"/>
+    </row>
+    <row r="83" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C83" s="1"/>
+    </row>
+    <row r="84" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C84" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1118,7 +1533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1127,7 +1542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1136,7 +1551,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1145,7 +1560,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1154,7 +1569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1351,7 +1766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add visualizations of profiling (latency)
</commit_message>
<xml_diff>
--- a/client-env/profiling/client_profiling.xlsx
+++ b/client-env/profiling/client_profiling.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\client-env\profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ADF53A2-C557-4C14-B92E-156F50CDD736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C5BF6BA-731C-4430-B362-0140DFF4732B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test_connection" sheetId="1" r:id="rId1"/>
     <sheet name="set" sheetId="9" r:id="rId2"/>
     <sheet name="get" sheetId="3" r:id="rId3"/>
     <sheet name="get_range" sheetId="4" r:id="rId4"/>
-    <sheet name="del_keys" sheetId="5" r:id="rId5"/>
+    <sheet name="delete" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>